<commit_message>
Did all required changes as per SOW before dedupe later, only data sources needed to be changed
</commit_message>
<xml_diff>
--- a/agent-3/outputs/agent3_dashboard.xlsx
+++ b/agent-3/outputs/agent3_dashboard.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,23 +99,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001565C0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="009E9E9E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="001F7A1F"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -190,6 +178,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
@@ -223,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -333,14 +327,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -349,6 +340,7 @@
     <xf numFmtId="0" fontId="12" fillId="13" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -357,6 +349,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -471,12 +466,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$12:$A$14</f>
+              <f>'Dashboard'!$A$12:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$12:$B$14</f>
+              <f>'Dashboard'!$B$12:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -1033,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1098,13 +1093,13 @@
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>FL, Florida</t>
+          <t>California, FL, Nebraska, New York, Texas</t>
         </is>
       </c>
       <c r="I2" s="4" t="n"/>
       <c r="J2" s="7" t="inlineStr">
         <is>
-          <t>22-Jun-2026 04:37 PM</t>
+          <t>22-Jun-2026 11:01 PM</t>
         </is>
       </c>
       <c r="K2" s="2" t="n"/>
@@ -1127,22 +1122,22 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Founder-Led:  5</t>
+          <t xml:space="preserve">  Founder-Led:  4</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Family-Owned:  4</t>
+          <t xml:space="preserve">  Family-Owned:  3</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Highest Score:  60</t>
+          <t xml:space="preserve">  Highest Score:  125</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Today:  2</t>
+          <t xml:space="preserve">  New Today:  11</t>
         </is>
       </c>
     </row>
@@ -1196,24 +1191,24 @@
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="22" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="23" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="17" t="n"/>
       <c r="G7" s="17" t="n"/>
       <c r="H7" s="25" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I7" s="19" t="n"/>
       <c r="J7" s="26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" s="21" t="n"/>
       <c r="L7" s="21" t="n"/>
@@ -1227,26 +1222,26 @@
       <c r="B8" s="13" t="n"/>
       <c r="C8" s="28" t="inlineStr">
         <is>
-          <t>vs Last Week: ↓ 5</t>
+          <t>vs Last Week: ↑ 5</t>
         </is>
       </c>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="29" t="inlineStr">
         <is>
-          <t>vs Last Week: ↑ 1</t>
+          <t>vs Last Week: — 0</t>
         </is>
       </c>
       <c r="F8" s="17" t="n"/>
       <c r="G8" s="17" t="n"/>
       <c r="H8" s="30" t="inlineStr">
         <is>
-          <t>vs Last Week: — 0</t>
+          <t>vs Last Week: ↑ 5</t>
         </is>
       </c>
       <c r="I8" s="19" t="n"/>
       <c r="J8" s="31" t="inlineStr">
         <is>
-          <t>vs Last Week: ↑ 2</t>
+          <t>vs Last Week: — 0</t>
         </is>
       </c>
       <c r="K8" s="21" t="n"/>
@@ -1306,11 +1301,11 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="32" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="B12" s="32" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" s="32" t="inlineStr">
         <is>
@@ -1322,15 +1317,15 @@
       </c>
       <c r="G12" s="32" t="inlineStr">
         <is>
-          <t>Medical Devices</t>
+          <t>Telecommunications</t>
         </is>
       </c>
       <c r="H12" s="32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="34" t="inlineStr">
         <is>
-          <t>• 56% of targets are founder-led</t>
+          <t>• 36% of targets are founder-led</t>
         </is>
       </c>
       <c r="L12" s="35" t="n"/>
@@ -1338,11 +1333,11 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="32" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B13" s="32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="32" t="inlineStr">
         <is>
@@ -1354,7 +1349,7 @@
       </c>
       <c r="G13" s="32" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Engines and Power Transm...</t>
         </is>
       </c>
       <c r="H13" s="32" t="n">
@@ -1366,7 +1361,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="32" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="B14" s="32" t="n">
@@ -1378,11 +1373,11 @@
         </is>
       </c>
       <c r="E14" s="32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="32" t="inlineStr">
         <is>
-          <t>Business Services &amp; Supp...</t>
+          <t>Individual and Family Se...</t>
         </is>
       </c>
       <c r="H14" s="32" t="n">
@@ -1390,23 +1385,31 @@
       </c>
       <c r="K14" s="34" t="inlineStr">
         <is>
-          <t>• 44% of targets are family-owned</t>
+          <t>• 27% of targets are family-owned</t>
         </is>
       </c>
       <c r="L14" s="35" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="D15" s="32" t="inlineStr">
         <is>
           <t>80-100</t>
         </is>
       </c>
       <c r="E15" s="32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="32" t="inlineStr">
         <is>
-          <t>Residential Building Con...</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="H15" s="32" t="n">
@@ -1416,9 +1419,17 @@
       <c r="L15" s="35" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="G16" s="32" t="inlineStr">
         <is>
-          <t>Venture Capital and Priv...</t>
+          <t>Transportation, Logistic...</t>
         </is>
       </c>
       <c r="H16" s="32" t="n">
@@ -1426,7 +1437,7 @@
       </c>
       <c r="K16" s="34" t="inlineStr">
         <is>
-          <t>• Florida has the highest volume</t>
+          <t>• FL has the highest volume</t>
         </is>
       </c>
       <c r="L16" s="35" t="n"/>
@@ -1438,7 +1449,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="K18" s="34" t="inlineStr">
         <is>
-          <t>• 2 new targets added this run</t>
+          <t>• 11 new targets added this run</t>
         </is>
       </c>
       <c r="L18" s="35" t="n"/>
@@ -1450,7 +1461,7 @@
     <row r="20" ht="16" customHeight="1">
       <c r="K20" s="34" t="inlineStr">
         <is>
-          <t>• 0 companies scored 80+</t>
+          <t>• 3 companies scored 80+</t>
         </is>
       </c>
       <c r="L20" s="35" t="n"/>
@@ -1533,43 +1544,43 @@
       </c>
       <c r="B29" s="38" t="inlineStr">
         <is>
-          <t>Arthrex</t>
+          <t>ATL Diesel</t>
         </is>
       </c>
       <c r="C29" s="38" t="inlineStr">
         <is>
-          <t>Reinhold Schmieding</t>
+          <t>Dan Bendever</t>
         </is>
       </c>
       <c r="D29" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>70-80</t>
         </is>
       </c>
       <c r="E29" s="40" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F29" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="G29" s="41" t="n">
-        <v>60</v>
+        <v>125</v>
       </c>
       <c r="H29" s="39" t="inlineStr">
         <is>
-          <t>Family-Owned, Founder-Led</t>
+          <t>Family-Owned</t>
         </is>
       </c>
       <c r="I29" s="42" t="inlineStr">
         <is>
-          <t>Pursuing</t>
+          <t>New</t>
         </is>
       </c>
       <c r="J29" s="38" t="inlineStr">
         <is>
-          <t>Arthrex's long history and family ownership make it an appealing acquisition target.</t>
+          <t>Established family-owned manufacturer with high seller readiness score.</t>
         </is>
       </c>
     </row>
@@ -1579,43 +1590,43 @@
       </c>
       <c r="B30" s="38" t="inlineStr">
         <is>
-          <t>American Sugar Refining</t>
+          <t>ATL Diesel</t>
         </is>
       </c>
       <c r="C30" s="38" t="inlineStr">
         <is>
-          <t>Florida Crystals Corporation and Sugar Cane Growers Cooperative of Florida</t>
+          <t>Dan Bendever</t>
         </is>
       </c>
       <c r="D30" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>70-80</t>
         </is>
       </c>
       <c r="E30" s="40" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="F30" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="G30" s="41" t="n">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="H30" s="39" t="inlineStr">
         <is>
-          <t>Family-Owned</t>
-        </is>
-      </c>
-      <c r="I30" s="43" t="inlineStr">
-        <is>
-          <t>Passed</t>
+          <t>Family-Owned, Founder-Led</t>
+        </is>
+      </c>
+      <c r="I30" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
         </is>
       </c>
       <c r="J30" s="38" t="inlineStr">
         <is>
-          <t>Established food industry player with strong family ownership and partnership structure.</t>
+          <t>Established company with high seller readiness and potential for acquisition.</t>
         </is>
       </c>
     </row>
@@ -1625,12 +1636,12 @@
       </c>
       <c r="B31" s="38" t="inlineStr">
         <is>
-          <t>Acosta</t>
+          <t>ALDI</t>
         </is>
       </c>
       <c r="C31" s="38" t="inlineStr">
         <is>
-          <t>L.T. Acosta</t>
+          <t>Karl and Theo Albrecht</t>
         </is>
       </c>
       <c r="D31" s="39" t="inlineStr">
@@ -1639,29 +1650,29 @@
         </is>
       </c>
       <c r="E31" s="40" t="n">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="F31" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="G31" s="44" t="n">
-        <v>35</v>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G31" s="41" t="n">
+        <v>85</v>
       </c>
       <c r="H31" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I31" s="45" t="inlineStr">
+          <t>Family-Owned</t>
+        </is>
+      </c>
+      <c r="I31" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J31" s="38" t="inlineStr">
         <is>
-          <t>Acosta's 99 years in business make it a stable acquisition target.</t>
+          <t>ALDI's strong family ownership and high seller readiness make it an attractive acquisition target.</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1682,12 @@
       </c>
       <c r="B32" s="38" t="inlineStr">
         <is>
-          <t>AG GENERAL CONTRACTOR</t>
+          <t>All Florida Paper</t>
         </is>
       </c>
       <c r="C32" s="38" t="inlineStr">
         <is>
-          <t>Guillermo Gaona and Pablo Allamand Sr.</t>
+          <t>Armando Caceres</t>
         </is>
       </c>
       <c r="D32" s="39" t="inlineStr">
@@ -1685,29 +1696,29 @@
         </is>
       </c>
       <c r="E32" s="40" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="F32" s="39" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="G32" s="44" t="n">
-        <v>35</v>
+      <c r="G32" s="43" t="n">
+        <v>45</v>
       </c>
       <c r="H32" s="39" t="inlineStr">
         <is>
           <t>Founder-Led</t>
         </is>
       </c>
-      <c r="I32" s="45" t="inlineStr">
+      <c r="I32" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J32" s="38" t="inlineStr">
         <is>
-          <t>Established contractor with strong leadership and 46 years of industry experience.</t>
+          <t>Established logistics company with 33 years of experience and moderate seller readiness.</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1728,7 @@
       </c>
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>AB Committed Capital</t>
+          <t>Acosta</t>
         </is>
       </c>
       <c r="C33" s="38" t="inlineStr">
@@ -1731,29 +1742,29 @@
         </is>
       </c>
       <c r="E33" s="40" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F33" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="G33" s="44" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H33" s="39" t="inlineStr">
         <is>
-          <t>Family-Owned</t>
-        </is>
-      </c>
-      <c r="I33" s="45" t="inlineStr">
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I33" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J33" s="38" t="inlineStr">
         <is>
-          <t>Strong acquisition target backed by successful family offices in private investment.</t>
+          <t>Acosta's long history and current leadership make it a compelling acquisition target.</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1774,12 @@
       </c>
       <c r="B34" s="38" t="inlineStr">
         <is>
-          <t>AB Committed Capital</t>
+          <t>Accordis International</t>
         </is>
       </c>
       <c r="C34" s="38" t="inlineStr">
         <is>
-          <t>Evan Bozymski, Nicholas Adam</t>
+          <t>Rehan Khan</t>
         </is>
       </c>
       <c r="D34" s="39" t="inlineStr">
@@ -1777,29 +1788,29 @@
         </is>
       </c>
       <c r="E34" s="40" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="F34" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="G34" s="44" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H34" s="39" t="inlineStr">
         <is>
-          <t>Family-Owned, Founder-Led</t>
-        </is>
-      </c>
-      <c r="I34" s="45" t="inlineStr">
+          <t>Founder-Led</t>
+        </is>
+      </c>
+      <c r="I34" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J34" s="38" t="inlineStr">
         <is>
-          <t>AB Committed Capital is a promising family-owned investment firm with strong leadership.</t>
+          <t>Accordis International is a stable, experienced IT services firm with founder-led leadership.</t>
         </is>
       </c>
     </row>
@@ -1809,12 +1820,12 @@
       </c>
       <c r="B35" s="38" t="inlineStr">
         <is>
-          <t>ALARM BROKERS OF FLORIDA LLC</t>
+          <t>Accordion Partners</t>
         </is>
       </c>
       <c r="C35" s="38" t="inlineStr">
         <is>
-          <t>Steve Carulo and Mary Runno</t>
+          <t>Nick Leopard</t>
         </is>
       </c>
       <c r="D35" s="39" t="inlineStr">
@@ -1823,29 +1834,29 @@
         </is>
       </c>
       <c r="E35" s="40" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F35" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="G35" s="44" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H35" s="39" t="inlineStr">
         <is>
           <t>Founder-Led</t>
         </is>
       </c>
-      <c r="I35" s="45" t="inlineStr">
+      <c r="I35" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J35" s="38" t="inlineStr">
         <is>
-          <t>Strong acquisition target with industry expertise and high seller readiness.</t>
+          <t>Accordion Partners is a seasoned consulting firm with strong leadership and growth potential.</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1866,12 @@
       </c>
       <c r="B36" s="38" t="inlineStr">
         <is>
-          <t>Air Pros USA</t>
+          <t>Allo</t>
         </is>
       </c>
       <c r="C36" s="38" t="inlineStr">
         <is>
-          <t>Anthony Perera</t>
+          <t>Brad Moline</t>
         </is>
       </c>
       <c r="D36" s="39" t="inlineStr">
@@ -1869,29 +1880,29 @@
         </is>
       </c>
       <c r="E36" s="40" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F36" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="G36" s="44" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H36" s="39" t="inlineStr">
         <is>
-          <t>Founder-Led</t>
-        </is>
-      </c>
-      <c r="I36" s="45" t="inlineStr">
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I36" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J36" s="38" t="inlineStr">
         <is>
-          <t>Air Pros USA is poised for growth under founder-led leadership.</t>
+          <t>Allo is a stable telecommunications company with a strong Seller Readiness Score.</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1912,12 @@
       </c>
       <c r="B37" s="38" t="inlineStr">
         <is>
-          <t>Altrius</t>
+          <t>Accelerate Capital Group</t>
         </is>
       </c>
       <c r="C37" s="38" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Alexis Graham, Ian Tracy</t>
         </is>
       </c>
       <c r="D37" s="39" t="inlineStr">
@@ -1915,29 +1926,121 @@
         </is>
       </c>
       <c r="E37" s="40" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="F37" s="39" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G37" s="44" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H37" s="39" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="I37" s="45" t="inlineStr">
+      <c r="I37" s="42" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
       <c r="J37" s="38" t="inlineStr">
         <is>
-          <t>Altrius is a young insurance company with growth potential in Florida.</t>
+          <t>Accelerate Capital Group is a stable financial services firm with high seller readiness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>2600Hz</t>
+        </is>
+      </c>
+      <c r="C38" s="38" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D38" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E38" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="F38" s="39" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="G38" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="H38" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I38" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J38" s="38" t="inlineStr">
+        <is>
+          <t>2600Hz is a prime acquisition target with a high seller readiness score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>Affinity Beverages LLC</t>
+        </is>
+      </c>
+      <c r="C39" s="38" t="inlineStr">
+        <is>
+          <t>Stanley Rottell</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E39" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="G39" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="H39" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I39" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J39" s="38" t="inlineStr">
+        <is>
+          <t>Affinity Beverages LLC shows strong acquisition potential with a high seller readiness score.</t>
         </is>
       </c>
     </row>
@@ -1991,7 +2094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2011,651 +2114,779 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" s="46" t="inlineStr">
+      <c r="B1" s="45" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="C1" s="46" t="inlineStr">
+      <c r="C1" s="45" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
       </c>
-      <c r="D1" s="46" t="inlineStr">
+      <c r="D1" s="45" t="inlineStr">
         <is>
           <t>Company Type</t>
         </is>
       </c>
-      <c r="E1" s="46" t="inlineStr">
+      <c r="E1" s="45" t="inlineStr">
         <is>
           <t>Founded Year</t>
         </is>
       </c>
-      <c r="F1" s="46" t="inlineStr">
+      <c r="F1" s="45" t="inlineStr">
         <is>
           <t>Years in Business</t>
         </is>
       </c>
-      <c r="G1" s="46" t="inlineStr">
+      <c r="G1" s="45" t="inlineStr">
         <is>
           <t>Founder Name</t>
         </is>
       </c>
-      <c r="H1" s="46" t="inlineStr">
+      <c r="H1" s="45" t="inlineStr">
         <is>
           <t>Founder Led</t>
         </is>
       </c>
-      <c r="I1" s="46" t="inlineStr">
+      <c r="I1" s="45" t="inlineStr">
         <is>
           <t>Family Owned</t>
         </is>
       </c>
-      <c r="J1" s="46" t="inlineStr">
+      <c r="J1" s="45" t="inlineStr">
         <is>
           <t>Founder Age Est.</t>
         </is>
       </c>
-      <c r="K1" s="46" t="inlineStr">
+      <c r="K1" s="45" t="inlineStr">
         <is>
           <t>Seller Readiness Score</t>
         </is>
       </c>
-      <c r="L1" s="46" t="inlineStr">
+      <c r="L1" s="45" t="inlineStr">
         <is>
           <t>Review Status</t>
         </is>
       </c>
-      <c r="M1" s="46" t="inlineStr">
+      <c r="M1" s="45" t="inlineStr">
         <is>
           <t>First Seen</t>
         </is>
       </c>
-      <c r="N1" s="46" t="inlineStr">
+      <c r="N1" s="45" t="inlineStr">
         <is>
           <t>Last Seen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47" t="inlineStr">
-        <is>
-          <t>Arthrex</t>
-        </is>
-      </c>
-      <c r="B2" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C2" s="47" t="inlineStr">
-        <is>
-          <t>Medical Devices</t>
-        </is>
-      </c>
-      <c r="D2" s="47" t="inlineStr">
+      <c r="A2" s="46" t="inlineStr">
+        <is>
+          <t>ATL Diesel</t>
+        </is>
+      </c>
+      <c r="B2" s="46" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="C2" s="46" t="inlineStr">
+        <is>
+          <t>Engines and Power Transmission Equipment Manufacturing</t>
+        </is>
+      </c>
+      <c r="D2" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E2" s="46" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="F2" s="46" t="n">
+        <v>53</v>
+      </c>
+      <c r="G2" s="46" t="inlineStr">
+        <is>
+          <t>Dan Bendever</t>
+        </is>
+      </c>
+      <c r="H2" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I2" s="46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" s="46" t="inlineStr">
+        <is>
+          <t>70-80</t>
+        </is>
+      </c>
+      <c r="K2" s="47" t="n">
+        <v>125</v>
+      </c>
+      <c r="L2" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M2" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N2" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="46" t="inlineStr">
+        <is>
+          <t>ATL Diesel</t>
+        </is>
+      </c>
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="C3" s="46" t="inlineStr">
+        <is>
+          <t>Individual and Family Services</t>
+        </is>
+      </c>
+      <c r="D3" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E3" s="46" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="F3" s="46" t="n">
+        <v>53</v>
+      </c>
+      <c r="G3" s="46" t="inlineStr">
+        <is>
+          <t>Dan Bendever</t>
+        </is>
+      </c>
+      <c r="H3" s="46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I3" s="46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" s="46" t="inlineStr">
+        <is>
+          <t>70-80</t>
+        </is>
+      </c>
+      <c r="K3" s="47" t="n">
+        <v>115</v>
+      </c>
+      <c r="L3" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M3" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N3" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>ALDI</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Private</t>
         </is>
       </c>
-      <c r="E2" s="47" t="inlineStr">
-        <is>
-          <t>1980</t>
-        </is>
-      </c>
-      <c r="F2" s="47" t="n">
-        <v>46</v>
-      </c>
-      <c r="G2" s="47" t="inlineStr">
-        <is>
-          <t>Reinhold Schmieding</t>
-        </is>
-      </c>
-      <c r="H2" s="47" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
+        <is>
+          <t>1946</t>
+        </is>
+      </c>
+      <c r="F4" s="46" t="n">
+        <v>80</v>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>Karl and Theo Albrecht</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I4" s="46" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I2" s="47" t="inlineStr">
+      <c r="J4" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K4" s="47" t="n">
+        <v>85</v>
+      </c>
+      <c r="L4" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M4" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N4" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>All Florida Paper</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>Transportation, Logistics, Supply Chain and Storage</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="n">
+        <v>33</v>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>Armando Caceres</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J2" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K2" s="48" t="n">
-        <v>60</v>
-      </c>
-      <c r="L2" s="47" t="inlineStr">
-        <is>
-          <t>Pursuing</t>
-        </is>
-      </c>
-      <c r="M2" s="49" t="n">
+      <c r="I5" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J5" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K5" s="49" t="n">
+        <v>45</v>
+      </c>
+      <c r="L5" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M5" s="48" t="n">
         <v>46195</v>
       </c>
-      <c r="N2" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>46195</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="47" t="inlineStr">
-        <is>
-          <t>American Sugar Refining</t>
-        </is>
-      </c>
-      <c r="B3" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C3" s="47" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="D3" s="47" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>Acosta</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>Business Services &amp; Supplies</t>
+        </is>
+      </c>
+      <c r="D6" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E6" s="46" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="F6" s="46" t="n">
+        <v>99</v>
+      </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J6" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K6" s="50" t="n">
+        <v>35</v>
+      </c>
+      <c r="L6" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M6" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N6" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>Accordis International</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>IT Services and IT Consulting</t>
+        </is>
+      </c>
+      <c r="D7" s="46" t="inlineStr">
         <is>
           <t>Private</t>
         </is>
       </c>
-      <c r="E3" s="47" t="inlineStr">
-        <is>
-          <t>1998</t>
-        </is>
-      </c>
-      <c r="F3" s="47" t="n">
-        <v>28</v>
-      </c>
-      <c r="G3" s="47" t="inlineStr">
-        <is>
-          <t>Florida Crystals Corporation and Sugar Cane Growers Cooperative of Florida</t>
-        </is>
-      </c>
-      <c r="H3" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I3" s="47" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="n">
+        <v>18</v>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>Rehan Khan</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J3" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K3" s="48" t="n">
-        <v>45</v>
-      </c>
-      <c r="L3" s="47" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="M3" s="49" t="n">
+      <c r="I7" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J7" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K7" s="50" t="n">
+        <v>35</v>
+      </c>
+      <c r="L7" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M7" s="48" t="n">
         <v>46195</v>
       </c>
-      <c r="N3" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>46195</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="47" t="inlineStr">
-        <is>
-          <t>Acosta</t>
-        </is>
-      </c>
-      <c r="B4" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C4" s="47" t="inlineStr">
-        <is>
-          <t>Business Services &amp; Supplies</t>
-        </is>
-      </c>
-      <c r="D4" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E4" s="47" t="inlineStr">
-        <is>
-          <t>1927</t>
-        </is>
-      </c>
-      <c r="F4" s="47" t="n">
-        <v>99</v>
-      </c>
-      <c r="G4" s="47" t="inlineStr">
-        <is>
-          <t>L.T. Acosta</t>
-        </is>
-      </c>
-      <c r="H4" s="47" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t>Accordion Partners</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>Consulting firm</t>
+        </is>
+      </c>
+      <c r="D8" s="46" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="n">
+        <v>17</v>
+      </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>Nick Leopard</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I8" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J8" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K8" s="50" t="n">
+        <v>25</v>
+      </c>
+      <c r="L8" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M8" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N8" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>Allo</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>Telecommunications</t>
+        </is>
+      </c>
+      <c r="D9" s="46" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="n">
+        <v>23</v>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>Brad Moline</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I4" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J4" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K4" s="50" t="n">
-        <v>35</v>
-      </c>
-      <c r="L4" s="47" t="inlineStr">
+      <c r="I9" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J9" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K9" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="L9" s="46" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="M4" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N4" s="49" t="n">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="47" t="inlineStr">
-        <is>
-          <t>AG GENERAL CONTRACTOR</t>
-        </is>
-      </c>
-      <c r="B5" s="47" t="inlineStr">
+      <c r="M9" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N9" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>Accelerate Capital Group</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="n">
+        <v>18</v>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
+        <is>
+          <t>Alexis Graham, Ian Tracy</t>
+        </is>
+      </c>
+      <c r="H10" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I10" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J10" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L10" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M10" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N10" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>2600Hz</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Telecommunications</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="F11" s="46" t="n">
+        <v>16</v>
+      </c>
+      <c r="G11" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J11" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K11" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M11" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N11" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>Affinity Beverages LLC</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="C5" s="47" t="inlineStr">
-        <is>
-          <t>Residential Building Construction</t>
-        </is>
-      </c>
-      <c r="D5" s="47" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E5" s="47" t="inlineStr">
-        <is>
-          <t>1980</t>
-        </is>
-      </c>
-      <c r="F5" s="47" t="n">
-        <v>46</v>
-      </c>
-      <c r="G5" s="47" t="inlineStr">
-        <is>
-          <t>Guillermo Gaona and Pablo Allamand Sr.</t>
-        </is>
-      </c>
-      <c r="H5" s="47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I5" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J5" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K5" s="50" t="n">
-        <v>35</v>
-      </c>
-      <c r="L5" s="47" t="inlineStr">
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="D12" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" s="46" t="inlineStr">
+        <is>
+          <t>Stanley Rottell</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I12" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J12" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K12" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L12" s="46" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="M5" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N5" s="49" t="n">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="47" t="inlineStr">
-        <is>
-          <t>AB Committed Capital</t>
-        </is>
-      </c>
-      <c r="B6" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C6" s="47" t="inlineStr">
-        <is>
-          <t>Venture Capital and Private Equity Principals</t>
-        </is>
-      </c>
-      <c r="D6" s="47" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E6" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F6" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H6" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I6" s="47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J6" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K6" s="50" t="n">
-        <v>25</v>
-      </c>
-      <c r="L6" s="47" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M6" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N6" s="49" t="n">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="47" t="inlineStr">
-        <is>
-          <t>AB Committed Capital</t>
-        </is>
-      </c>
-      <c r="B7" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C7" s="47" t="inlineStr">
-        <is>
-          <t>Investment</t>
-        </is>
-      </c>
-      <c r="D7" s="47" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E7" s="47" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="F7" s="47" t="n">
-        <v>3</v>
-      </c>
-      <c r="G7" s="47" t="inlineStr">
-        <is>
-          <t>Evan Bozymski, Nicholas Adam</t>
-        </is>
-      </c>
-      <c r="H7" s="47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I7" s="47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J7" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K7" s="50" t="n">
-        <v>25</v>
-      </c>
-      <c r="L7" s="47" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M7" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N7" s="49" t="n">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="47" t="inlineStr">
-        <is>
-          <t>ALARM BROKERS OF FLORIDA LLC</t>
-        </is>
-      </c>
-      <c r="B8" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C8" s="47" t="inlineStr">
-        <is>
-          <t>Security and Investigations</t>
-        </is>
-      </c>
-      <c r="D8" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E8" s="47" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="F8" s="47" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" s="47" t="inlineStr">
-        <is>
-          <t>Steve Carulo and Mary Runno</t>
-        </is>
-      </c>
-      <c r="H8" s="47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I8" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J8" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K8" s="50" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="47" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M8" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N8" s="49" t="n">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="47" t="inlineStr">
-        <is>
-          <t>Air Pros USA</t>
-        </is>
-      </c>
-      <c r="B9" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C9" s="47" t="inlineStr">
-        <is>
-          <t>HVAC and Refrigeration Equipment Manufacturing</t>
-        </is>
-      </c>
-      <c r="D9" s="47" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="E9" s="47" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="F9" s="47" t="n">
-        <v>9</v>
-      </c>
-      <c r="G9" s="47" t="inlineStr">
-        <is>
-          <t>Anthony Perera</t>
-        </is>
-      </c>
-      <c r="H9" s="47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I9" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J9" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K9" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="47" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M9" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N9" s="49" t="n">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="47" t="inlineStr">
-        <is>
-          <t>Altrius</t>
-        </is>
-      </c>
-      <c r="B10" s="47" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
-      </c>
-      <c r="C10" s="47" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="D10" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E10" s="47" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="F10" s="47" t="n">
-        <v>6</v>
-      </c>
-      <c r="G10" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H10" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I10" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J10" s="47" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="K10" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="47" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="M10" s="49" t="n">
-        <v>46194</v>
-      </c>
-      <c r="N10" s="49" t="n">
-        <v>46194</v>
+      <c r="M12" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N12" s="48" t="n">
+        <v>46195</v>
       </c>
     </row>
   </sheetData>
@@ -2670,7 +2901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2686,52 +2917,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B1" s="46" t="inlineStr">
+      <c r="B1" s="45" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="C1" s="46" t="inlineStr">
+      <c r="C1" s="45" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="D1" s="46" t="inlineStr">
+      <c r="D1" s="45" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="E1" s="46" t="inlineStr">
+      <c r="E1" s="45" t="inlineStr">
         <is>
           <t>Why Selected</t>
         </is>
       </c>
-      <c r="F1" s="46" t="inlineStr">
+      <c r="F1" s="45" t="inlineStr">
         <is>
           <t>Evidence Summary</t>
         </is>
       </c>
-      <c r="G1" s="46" t="inlineStr">
+      <c r="G1" s="45" t="inlineStr">
         <is>
           <t>One-line Reason</t>
         </is>
       </c>
-      <c r="H1" s="46" t="inlineStr">
+      <c r="H1" s="45" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="I1" s="46" t="inlineStr">
+      <c r="I1" s="45" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="J1" s="46" t="inlineStr">
+      <c r="J1" s="45" t="inlineStr">
         <is>
           <t>_candidate_id</t>
         </is>
@@ -2743,40 +2974,40 @@
       </c>
       <c r="B2" s="52" t="inlineStr">
         <is>
-          <t>Arthrex</t>
+          <t>ATL Diesel</t>
         </is>
       </c>
       <c r="C2" s="53" t="n">
-        <v>60</v>
+        <v>125</v>
       </c>
       <c r="D2" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="E2" s="52" t="inlineStr">
         <is>
-          <t>Arthrex is a strong acquisition target due to its long-standing presence in the medical devices industry, having been in business for 46 years. The company's family-owned structure and founder-led management may provide stability and a unique culture that could be attractive to potential buyers.</t>
+          <t>ATL Diesel is a well-established company with 53 years in the engines and power transmission equipment manufacturing industry. Its family-owned status and high seller readiness score of 125 indicate a strong potential for acquisition, especially as the founder approaches retirement age.</t>
         </is>
       </c>
       <c r="F2" s="52" t="inlineStr">
         <is>
-          <t>The evidence indicates that Arthrex was founded in 1980 by Reinhold Schmieding, who is still leading the company as President, and it is described as a privately held family business.</t>
+          <t>The evidence supporting this selection is limited, but the high seller readiness score and the company's long history suggest a favorable acquisition opportunity.</t>
         </is>
       </c>
       <c r="G2" s="52" t="inlineStr">
         <is>
-          <t>Arthrex's long history and family ownership make it an appealing acquisition target.</t>
+          <t>Established family-owned manufacturer with high seller readiness score.</t>
         </is>
       </c>
       <c r="H2" s="52" t="inlineStr">
         <is>
-          <t>Pursuing</t>
+          <t>New</t>
         </is>
       </c>
       <c r="I2" s="52" t="inlineStr"/>
       <c r="J2" s="52" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1">
@@ -2785,40 +3016,40 @@
       </c>
       <c r="B3" s="52" t="inlineStr">
         <is>
-          <t>American Sugar Refining</t>
+          <t>ATL Diesel</t>
         </is>
       </c>
       <c r="C3" s="53" t="n">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="D3" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E3" s="52" t="inlineStr">
         <is>
-          <t>American Sugar Refining is a strong acquisition target due to its established presence in the food industry and its long history of 28 years in business. The company's family-owned structure and partnership with the Sugar Cane Growers Cooperative of Florida suggest stability and potential for strategic growth.</t>
+          <t>ATL Diesel is a well-established company with 53 years in the Individual and Family Services industry, indicating stability and experience. The founder, Dan Bendever, is likely nearing retirement age, which may motivate a sale, and the high seller readiness score of 115 suggests the company is prepared for acquisition.</t>
         </is>
       </c>
       <c r="F3" s="52" t="inlineStr">
         <is>
-          <t>The company is part of a larger sugar empire owned by the Fanjul brothers, with origins in 19th-century sugar plantations, indicating a deep-rooted legacy in the industry. However, specific details about the founder's leadership and readiness for sale are limited.</t>
+          <t>The evidence is limited, but the company's long history and high seller readiness score support its selection as an acquisition target.</t>
         </is>
       </c>
       <c r="G3" s="52" t="inlineStr">
         <is>
-          <t>Established food industry player with strong family ownership and partnership structure.</t>
+          <t>Established company with high seller readiness and potential for acquisition.</t>
         </is>
       </c>
       <c r="H3" s="52" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>New</t>
         </is>
       </c>
       <c r="I3" s="52" t="inlineStr"/>
       <c r="J3" s="52" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" ht="90" customHeight="1">
@@ -2827,30 +3058,30 @@
       </c>
       <c r="B4" s="52" t="inlineStr">
         <is>
-          <t>Acosta</t>
-        </is>
-      </c>
-      <c r="C4" s="54" t="n">
-        <v>35</v>
+          <t>ALDI</t>
+        </is>
+      </c>
+      <c r="C4" s="53" t="n">
+        <v>85</v>
       </c>
       <c r="D4" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E4" s="52" t="inlineStr">
         <is>
-          <t>Acosta is a well-established company with 99 years in the business services and supplies industry, indicating stability and experience. The current leadership under CEO Darian Pickett suggests a potential for growth and innovation, making it an attractive acquisition target.</t>
+          <t>ALDI is a strong acquisition target due to its long-standing family ownership and high seller readiness score of 85, indicating a favorable disposition towards potential buyers. With 80 years in the retail industry, ALDI has established a solid market presence and brand loyalty.</t>
         </is>
       </c>
       <c r="F4" s="52" t="inlineStr">
         <is>
-          <t>Founded in 1927 as L.T. Acosta Co. Inc. in Jacksonville, the company has a long history, although the seller readiness score of 35 indicates some challenges in readiness for sale.</t>
+          <t>The company was founded by Karl and Theo Albrecht in 1946 and has remained family-owned, with a significant seller readiness score of 85. The split into two groups in 1960 further emphasizes the continuity of family ownership.</t>
         </is>
       </c>
       <c r="G4" s="52" t="inlineStr">
         <is>
-          <t>Acosta's 99 years in business make it a stable acquisition target.</t>
+          <t>ALDI's strong family ownership and high seller readiness make it an attractive acquisition target.</t>
         </is>
       </c>
       <c r="H4" s="52" t="inlineStr">
@@ -2860,7 +3091,7 @@
       </c>
       <c r="I4" s="52" t="inlineStr"/>
       <c r="J4" s="52" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" ht="90" customHeight="1">
@@ -2869,11 +3100,11 @@
       </c>
       <c r="B5" s="52" t="inlineStr">
         <is>
-          <t>AG GENERAL CONTRACTOR</t>
+          <t>All Florida Paper</t>
         </is>
       </c>
       <c r="C5" s="54" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D5" s="52" t="inlineStr">
         <is>
@@ -2882,17 +3113,17 @@
       </c>
       <c r="E5" s="52" t="inlineStr">
         <is>
-          <t>AG General Contractor is a well-established company with 46 years in the residential building construction industry, indicating stability and experience. The founder-led structure suggests strong leadership and continuity, which can be attractive to potential acquirers.</t>
+          <t>All Florida Paper has a long-standing presence in the transportation, logistics, supply chain, and storage industry, having been founded in 1993. With 33 years in business, the company demonstrates stability and experience, making it a potentially attractive acquisition target.</t>
         </is>
       </c>
       <c r="F5" s="52" t="inlineStr">
         <is>
-          <t>The company was founded in 1980 by Guillermo Gaona and Pablo Allamand Sr., and Pablo Allamand is currently listed as the registered agent and holds a managerial position, indicating ongoing founder involvement.</t>
+          <t>The Seller Readiness Score of 45 indicates a moderate level of preparedness for a sale, although no additional evidence is provided to further support this selection.</t>
         </is>
       </c>
       <c r="G5" s="52" t="inlineStr">
         <is>
-          <t>Established contractor with strong leadership and 46 years of industry experience.</t>
+          <t>Established logistics company with 33 years of experience and moderate seller readiness.</t>
         </is>
       </c>
       <c r="H5" s="52" t="inlineStr">
@@ -2902,7 +3133,7 @@
       </c>
       <c r="I5" s="52" t="inlineStr"/>
       <c r="J5" s="52" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" ht="90" customHeight="1">
@@ -2911,30 +3142,30 @@
       </c>
       <c r="B6" s="52" t="inlineStr">
         <is>
-          <t>AB Committed Capital</t>
-        </is>
-      </c>
-      <c r="C6" s="54" t="n">
-        <v>25</v>
+          <t>Acosta</t>
+        </is>
+      </c>
+      <c r="C6" s="55" t="n">
+        <v>35</v>
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E6" s="52" t="inlineStr">
         <is>
-          <t>AB Committed Capital is a strong acquisition target due to its backing from multiple family offices, indicating a solid financial foundation and potential for growth. Additionally, its focus on private investment positions it well within the venture capital and private equity industry.</t>
+          <t>Acosta is a well-established company with 99 years in the business services and supplies industry, indicating stability and experience. The current leadership under CEO Darian Pickett suggests a potential for continued growth and innovation, making it an attractive acquisition target.</t>
         </is>
       </c>
       <c r="F6" s="52" t="inlineStr">
         <is>
-          <t>The evidence indicates that AB Committed Capital is supported by successful operators through family offices, although specific details about the company, such as its founding year and leadership, are limited.</t>
+          <t>Acosta Sales &amp; Marketing was founded in 1927, and the current CEO is Darian Pickett, indicating a strong leadership structure. However, details about family ownership and the founder's background are limited.</t>
         </is>
       </c>
       <c r="G6" s="52" t="inlineStr">
         <is>
-          <t>Strong acquisition target backed by successful family offices in private investment.</t>
+          <t>Acosta's long history and current leadership make it a compelling acquisition target.</t>
         </is>
       </c>
       <c r="H6" s="52" t="inlineStr">
@@ -2944,7 +3175,7 @@
       </c>
       <c r="I6" s="52" t="inlineStr"/>
       <c r="J6" s="52" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="90" customHeight="1">
@@ -2953,30 +3184,30 @@
       </c>
       <c r="B7" s="52" t="inlineStr">
         <is>
-          <t>AB Committed Capital</t>
-        </is>
-      </c>
-      <c r="C7" s="54" t="n">
-        <v>25</v>
+          <t>Accordis International</t>
+        </is>
+      </c>
+      <c r="C7" s="55" t="n">
+        <v>35</v>
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E7" s="52" t="inlineStr">
         <is>
-          <t>AB Committed Capital is a relatively new investment firm with a strong family ownership structure, which may appeal to buyers looking for stable, long-term investments. The company's leadership by founders Evan Bozymski and Nicholas Adam suggests a committed management team that could facilitate a smooth transition post-acquisition.</t>
+          <t>Accordis International has been in business for 18 years, indicating stability and experience in the IT Services and IT Consulting industry. The founder-led structure may provide a strong vision and leadership continuity, making it an attractive acquisition target.</t>
         </is>
       </c>
       <c r="F7" s="52" t="inlineStr">
         <is>
-          <t>The company was founded in 2023 and is backed by multiple family offices, indicating it is family-owned. Additionally, the leadership roles of the founders provide a solid foundation for potential growth.</t>
+          <t>The evidence is limited, with no additional information captured, but the company's long tenure and founder-led status support its potential as an acquisition target.</t>
         </is>
       </c>
       <c r="G7" s="52" t="inlineStr">
         <is>
-          <t>AB Committed Capital is a promising family-owned investment firm with strong leadership.</t>
+          <t>Accordis International is a stable, experienced IT services firm with founder-led leadership.</t>
         </is>
       </c>
       <c r="H7" s="52" t="inlineStr">
@@ -2986,7 +3217,7 @@
       </c>
       <c r="I7" s="52" t="inlineStr"/>
       <c r="J7" s="52" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1">
@@ -2995,30 +3226,30 @@
       </c>
       <c r="B8" s="52" t="inlineStr">
         <is>
-          <t>ALARM BROKERS OF FLORIDA LLC</t>
-        </is>
-      </c>
-      <c r="C8" s="54" t="n">
-        <v>10</v>
+          <t>Accordion Partners</t>
+        </is>
+      </c>
+      <c r="C8" s="55" t="n">
+        <v>25</v>
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E8" s="52" t="inlineStr">
         <is>
-          <t>Alarm Brokers of Florida LLC is a strong acquisition target due to its solid foundation in the security and investigations industry, established by experienced founders. With a high seller readiness score of 10, the company is well-prepared for acquisition.</t>
+          <t>Accordion Partners is a well-established consulting firm with 17 years in business, led by its founder Nick Leopard. The company's private status and the founder's active role as CEO suggest potential for strategic growth and alignment with acquisition goals.</t>
         </is>
       </c>
       <c r="F8" s="52" t="inlineStr">
         <is>
-          <t>The company was founded by industry experts Steve Carulo and Mary Runno in 2016, and it has been in business for 10 years, indicating stability and expertise.</t>
+          <t>The company was founded in 2009 by Nick Leopard, who currently serves as CEO and Founder, indicating strong leadership. However, evidence regarding family ownership and the founder's age is limited.</t>
         </is>
       </c>
       <c r="G8" s="52" t="inlineStr">
         <is>
-          <t>Strong acquisition target with industry expertise and high seller readiness.</t>
+          <t>Accordion Partners is a seasoned consulting firm with strong leadership and growth potential.</t>
         </is>
       </c>
       <c r="H8" s="52" t="inlineStr">
@@ -3028,7 +3259,7 @@
       </c>
       <c r="I8" s="52" t="inlineStr"/>
       <c r="J8" s="52" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
@@ -3037,30 +3268,30 @@
       </c>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>Air Pros USA</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="n">
-        <v>0</v>
+          <t>Allo</t>
+        </is>
+      </c>
+      <c r="C9" s="55" t="n">
+        <v>20</v>
       </c>
       <c r="D9" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="E9" s="52" t="inlineStr">
         <is>
-          <t>Air Pros USA is a strong acquisition target due to its recent reacquisition by founder Anthony Perera, indicating a commitment to revitalizing the company. With 9 years in the HVAC and Refrigeration Equipment Manufacturing industry, it has established a foundation for growth under experienced leadership.</t>
+          <t>Allo is a well-established telecommunications company with 23 years in business, indicating stability and experience in the industry. Its Seller Readiness Score of 20 suggests a potential willingness to engage in acquisition discussions.</t>
         </is>
       </c>
       <c r="F9" s="52" t="inlineStr">
         <is>
-          <t>The evidence indicates that Air Pros USA was founded in 2017 by Anthony Perera, who has recently reacquired the company, suggesting a strategic move to enhance its market position.</t>
+          <t>Evidence is limited, but the company's long history and Seller Readiness Score support its selection as an acquisition target.</t>
         </is>
       </c>
       <c r="G9" s="52" t="inlineStr">
         <is>
-          <t>Air Pros USA is poised for growth under founder-led leadership.</t>
+          <t>Allo is a stable telecommunications company with a strong Seller Readiness Score.</t>
         </is>
       </c>
       <c r="H9" s="52" t="inlineStr">
@@ -3070,7 +3301,7 @@
       </c>
       <c r="I9" s="52" t="inlineStr"/>
       <c r="J9" s="52" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1">
@@ -3079,30 +3310,30 @@
       </c>
       <c r="B10" s="52" t="inlineStr">
         <is>
-          <t>Altrius</t>
-        </is>
-      </c>
-      <c r="C10" s="54" t="n">
-        <v>0</v>
+          <t>Accelerate Capital Group</t>
+        </is>
+      </c>
+      <c r="C10" s="55" t="n">
+        <v>10</v>
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E10" s="52" t="inlineStr">
         <is>
-          <t>Altrius, a relatively new player in the insurance industry, has potential for growth given its recent establishment in 2020 and small team size. Its location in West Palm Beach, Florida, may also provide strategic advantages in a competitive market.</t>
+          <t>Accelerate Capital Group has been in business for 18 years, indicating stability and experience in the financial services industry. The company has a high seller readiness score of 10, suggesting that it is well-prepared for acquisition discussions.</t>
         </is>
       </c>
       <c r="F10" s="52" t="inlineStr">
         <is>
-          <t>Altrius Group was founded in 2020 and has a small employee base of 2-10, indicating a startup phase with room for expansion. However, the seller readiness score is 0, suggesting limited immediate availability for acquisition.</t>
+          <t>The evidence is limited, but the company's long tenure and high seller readiness score support its selection as an acquisition target.</t>
         </is>
       </c>
       <c r="G10" s="52" t="inlineStr">
         <is>
-          <t>Altrius is a young insurance company with growth potential in Florida.</t>
+          <t>Accelerate Capital Group is a stable financial services firm with high seller readiness.</t>
         </is>
       </c>
       <c r="H10" s="52" t="inlineStr">
@@ -3112,12 +3343,54 @@
       </c>
       <c r="I10" s="52" t="inlineStr"/>
       <c r="J10" s="52" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="52" t="inlineStr">
+        <is>
+          <t>2600Hz</t>
+        </is>
+      </c>
+      <c r="C11" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="52" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="E11" s="52" t="inlineStr">
+        <is>
+          <t>2600Hz is a strong acquisition target due to its established presence in the telecommunications industry, having been in business for 16 years. The company's high seller readiness score of 10 indicates a strong willingness to engage in a sale, making it an attractive option for potential buyers.</t>
+        </is>
+      </c>
+      <c r="F11" s="52" t="inlineStr">
+        <is>
+          <t>The evidence supporting this selection is limited, but the high seller readiness score of 10 is a significant indicator of the company's preparedness for acquisition.</t>
+        </is>
+      </c>
+      <c r="G11" s="52" t="inlineStr">
+        <is>
+          <t>2600Hz is a prime acquisition target with a high seller readiness score.</t>
+        </is>
+      </c>
+      <c r="H11" s="52" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="I11" s="52" t="inlineStr"/>
+      <c r="J11" s="52" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Pursuing,Passed,Bad Data"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
made common .env for all agents, added agent 3 input search.
</commit_message>
<xml_diff>
--- a/agent-3/outputs/agent3_dashboard.xlsx
+++ b/agent-3/outputs/agent3_dashboard.xlsx
@@ -1028,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1099,7 +1099,7 @@
       <c r="I2" s="4" t="n"/>
       <c r="J2" s="7" t="inlineStr">
         <is>
-          <t>22-Jun-2026 11:01 PM</t>
+          <t>23-Jun-2026 04:52 PM</t>
         </is>
       </c>
       <c r="K2" s="2" t="n"/>
@@ -1122,7 +1122,7 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Founder-Led:  4</t>
+          <t xml:space="preserve">  Founder-Led:  7</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Today:  11</t>
+          <t xml:space="preserve">  New Today:  4</t>
         </is>
       </c>
     </row>
@@ -1191,11 +1191,11 @@
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="22" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="23" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="24" t="n">
@@ -1204,7 +1204,7 @@
       <c r="F7" s="17" t="n"/>
       <c r="G7" s="17" t="n"/>
       <c r="H7" s="25" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I7" s="19" t="n"/>
       <c r="J7" s="26" t="n">
@@ -1222,7 +1222,7 @@
       <c r="B8" s="13" t="n"/>
       <c r="C8" s="28" t="inlineStr">
         <is>
-          <t>vs Last Week: ↑ 5</t>
+          <t>vs Last Week: ↓ 2</t>
         </is>
       </c>
       <c r="D8" s="15" t="n"/>
@@ -1235,7 +1235,7 @@
       <c r="G8" s="17" t="n"/>
       <c r="H8" s="30" t="inlineStr">
         <is>
-          <t>vs Last Week: ↑ 5</t>
+          <t>vs Last Week: ↑ 9</t>
         </is>
       </c>
       <c r="I8" s="19" t="n"/>
@@ -1305,15 +1305,15 @@
         </is>
       </c>
       <c r="B12" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>20-40</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="n">
         <v>5</v>
-      </c>
-      <c r="D12" s="32" t="inlineStr">
-        <is>
-          <t>20-40</t>
-        </is>
-      </c>
-      <c r="E12" s="32" t="n">
-        <v>4</v>
       </c>
       <c r="G12" s="32" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="K12" s="34" t="inlineStr">
         <is>
-          <t>• 36% of targets are founder-led</t>
+          <t>• 47% of targets are founder-led</t>
         </is>
       </c>
       <c r="L12" s="35" t="n"/>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="B13" s="32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="32" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="E13" s="32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G13" s="32" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="K14" s="34" t="inlineStr">
         <is>
-          <t>• 27% of targets are family-owned</t>
+          <t>• 20% of targets are family-owned</t>
         </is>
       </c>
       <c r="L14" s="35" t="n"/>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G16" s="32" t="inlineStr">
         <is>
-          <t>Transportation, Logistic...</t>
+          <t>Warehousing and Storage</t>
         </is>
       </c>
       <c r="H16" s="32" t="n">
@@ -1449,7 +1449,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="K18" s="34" t="inlineStr">
         <is>
-          <t>• 11 new targets added this run</t>
+          <t>• 4 new targets added this run</t>
         </is>
       </c>
       <c r="L18" s="35" t="n"/>
@@ -1682,12 +1682,12 @@
       </c>
       <c r="B32" s="38" t="inlineStr">
         <is>
-          <t>All Florida Paper</t>
+          <t>AMWAT Moving Warehousing Storage</t>
         </is>
       </c>
       <c r="C32" s="38" t="inlineStr">
         <is>
-          <t>Armando Caceres</t>
+          <t>Gloria Maria Pugh</t>
         </is>
       </c>
       <c r="D32" s="39" t="inlineStr">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="E32" s="40" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F32" s="39" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="G32" s="43" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H32" s="39" t="inlineStr">
         <is>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="J32" s="38" t="inlineStr">
         <is>
-          <t>Established logistics company with 33 years of experience and moderate seller readiness.</t>
+          <t>Established warehousing company with over 25 years of operational experience.</t>
         </is>
       </c>
     </row>
@@ -1728,12 +1728,12 @@
       </c>
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>Acosta</t>
+          <t>All Florida Paper</t>
         </is>
       </c>
       <c r="C33" s="38" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Armando Caceres</t>
         </is>
       </c>
       <c r="D33" s="39" t="inlineStr">
@@ -1742,19 +1742,19 @@
         </is>
       </c>
       <c r="E33" s="40" t="n">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="F33" s="39" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="G33" s="44" t="n">
-        <v>35</v>
+      <c r="G33" s="43" t="n">
+        <v>45</v>
       </c>
       <c r="H33" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Founder-Led</t>
         </is>
       </c>
       <c r="I33" s="42" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="J33" s="38" t="inlineStr">
         <is>
-          <t>Acosta's long history and current leadership make it a compelling acquisition target.</t>
+          <t>Established logistics company with 33 years of experience and moderate seller readiness.</t>
         </is>
       </c>
     </row>
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B34" s="38" t="inlineStr">
         <is>
-          <t>Accordis International</t>
+          <t>Alternalight llc</t>
         </is>
       </c>
       <c r="C34" s="38" t="inlineStr">
         <is>
-          <t>Rehan Khan</t>
+          <t>Russell Stidolph</t>
         </is>
       </c>
       <c r="D34" s="39" t="inlineStr">
@@ -1788,15 +1788,15 @@
         </is>
       </c>
       <c r="E34" s="40" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F34" s="39" t="inlineStr">
         <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="G34" s="44" t="n">
-        <v>35</v>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G34" s="43" t="n">
+        <v>45</v>
       </c>
       <c r="H34" s="39" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="J34" s="38" t="inlineStr">
         <is>
-          <t>Accordis International is a stable, experienced IT services firm with founder-led leadership.</t>
+          <t>Alternalight LLC offers 20 years of experience in alternative energy under strong founder leadership.</t>
         </is>
       </c>
     </row>
@@ -1820,12 +1820,12 @@
       </c>
       <c r="B35" s="38" t="inlineStr">
         <is>
-          <t>Accordion Partners</t>
+          <t>Ameritape, Inc.</t>
         </is>
       </c>
       <c r="C35" s="38" t="inlineStr">
         <is>
-          <t>Nick Leopard</t>
+          <t>Renee Soares, Tom Whipple</t>
         </is>
       </c>
       <c r="D35" s="39" t="inlineStr">
@@ -1834,19 +1834,19 @@
         </is>
       </c>
       <c r="E35" s="40" t="n">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="F35" s="39" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="G35" s="44" t="n">
-        <v>25</v>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="G35" s="43" t="n">
+        <v>40</v>
       </c>
       <c r="H35" s="39" t="inlineStr">
         <is>
-          <t>Founder-Led</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="I35" s="42" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="J35" s="38" t="inlineStr">
         <is>
-          <t>Accordion Partners is a seasoned consulting firm with strong leadership and growth potential.</t>
+          <t>Ameritape, Inc. is a stable, niche player in automation machinery manufacturing.</t>
         </is>
       </c>
     </row>
@@ -1866,12 +1866,12 @@
       </c>
       <c r="B36" s="38" t="inlineStr">
         <is>
-          <t>Allo</t>
+          <t>Accordis International</t>
         </is>
       </c>
       <c r="C36" s="38" t="inlineStr">
         <is>
-          <t>Brad Moline</t>
+          <t>Rehan Khan</t>
         </is>
       </c>
       <c r="D36" s="39" t="inlineStr">
@@ -1880,19 +1880,19 @@
         </is>
       </c>
       <c r="E36" s="40" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F36" s="39" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="G36" s="44" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="H36" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Founder-Led</t>
         </is>
       </c>
       <c r="I36" s="42" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="J36" s="38" t="inlineStr">
         <is>
-          <t>Allo is a stable telecommunications company with a strong Seller Readiness Score.</t>
+          <t>Accordis International is a stable, experienced IT services firm with founder-led leadership.</t>
         </is>
       </c>
     </row>
@@ -1912,12 +1912,12 @@
       </c>
       <c r="B37" s="38" t="inlineStr">
         <is>
-          <t>Accelerate Capital Group</t>
+          <t>Acosta</t>
         </is>
       </c>
       <c r="C37" s="38" t="inlineStr">
         <is>
-          <t>Alexis Graham, Ian Tracy</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D37" s="39" t="inlineStr">
@@ -1926,15 +1926,15 @@
         </is>
       </c>
       <c r="E37" s="40" t="n">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="F37" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="G37" s="44" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="H37" s="39" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="J37" s="38" t="inlineStr">
         <is>
-          <t>Accelerate Capital Group is a stable financial services firm with high seller readiness.</t>
+          <t>Acosta's long history and current leadership make it a compelling acquisition target.</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="B38" s="38" t="inlineStr">
         <is>
-          <t>2600Hz</t>
+          <t>AirQuest Environmental, Inc.</t>
         </is>
       </c>
       <c r="C38" s="38" t="inlineStr">
@@ -1972,19 +1972,19 @@
         </is>
       </c>
       <c r="E38" s="40" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F38" s="39" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="G38" s="44" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="H38" s="39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Founder-Led</t>
         </is>
       </c>
       <c r="I38" s="42" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="J38" s="38" t="inlineStr">
         <is>
-          <t>2600Hz is a prime acquisition target with a high seller readiness score.</t>
+          <t>Established environmental services firm with 24 years of niche expertise.</t>
         </is>
       </c>
     </row>
@@ -2004,43 +2004,227 @@
       </c>
       <c r="B39" s="38" t="inlineStr">
         <is>
+          <t>Accordion Partners</t>
+        </is>
+      </c>
+      <c r="C39" s="38" t="inlineStr">
+        <is>
+          <t>Nick Leopard</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E39" s="40" t="n">
+        <v>17</v>
+      </c>
+      <c r="F39" s="39" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="G39" s="44" t="n">
+        <v>25</v>
+      </c>
+      <c r="H39" s="39" t="inlineStr">
+        <is>
+          <t>Founder-Led</t>
+        </is>
+      </c>
+      <c r="I39" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J39" s="38" t="inlineStr">
+        <is>
+          <t>Accordion Partners is a seasoned consulting firm with strong leadership and growth potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="37" t="n">
+        <v>12</v>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>Allo</t>
+        </is>
+      </c>
+      <c r="C40" s="38" t="inlineStr">
+        <is>
+          <t>Brad Moline</t>
+        </is>
+      </c>
+      <c r="D40" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E40" s="40" t="n">
+        <v>23</v>
+      </c>
+      <c r="F40" s="39" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
+      </c>
+      <c r="G40" s="44" t="n">
+        <v>20</v>
+      </c>
+      <c r="H40" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I40" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J40" s="38" t="inlineStr">
+        <is>
+          <t>Allo is a stable telecommunications company with a strong Seller Readiness Score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="37" t="n">
+        <v>13</v>
+      </c>
+      <c r="B41" s="38" t="inlineStr">
+        <is>
           <t>Affinity Beverages LLC</t>
         </is>
       </c>
-      <c r="C39" s="38" t="inlineStr">
+      <c r="C41" s="38" t="inlineStr">
         <is>
           <t>Stanley Rottell</t>
         </is>
       </c>
-      <c r="D39" s="39" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E39" s="40" t="n">
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E41" s="40" t="n">
         <v>12</v>
       </c>
-      <c r="F39" s="39" t="inlineStr">
+      <c r="F41" s="39" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="G39" s="44" t="n">
+      <c r="G41" s="44" t="n">
         <v>10</v>
       </c>
-      <c r="H39" s="39" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I39" s="42" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J39" s="38" t="inlineStr">
+      <c r="H41" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I41" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J41" s="38" t="inlineStr">
         <is>
           <t>Affinity Beverages LLC shows strong acquisition potential with a high seller readiness score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="37" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" s="38" t="inlineStr">
+        <is>
+          <t>Accelerate Capital Group</t>
+        </is>
+      </c>
+      <c r="C42" s="38" t="inlineStr">
+        <is>
+          <t>Alexis Graham, Ian Tracy</t>
+        </is>
+      </c>
+      <c r="D42" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E42" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="F42" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G42" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="H42" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I42" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J42" s="38" t="inlineStr">
+        <is>
+          <t>Accelerate Capital Group is a stable financial services firm with high seller readiness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>2600Hz</t>
+        </is>
+      </c>
+      <c r="C43" s="38" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D43" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E43" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="F43" s="39" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="G43" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="H43" s="39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I43" s="42" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="J43" s="38" t="inlineStr">
+        <is>
+          <t>2600Hz is a prime acquisition target with a high seller readiness score.</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2380,7 +2564,7 @@
     <row r="5">
       <c r="A5" s="46" t="inlineStr">
         <is>
-          <t>All Florida Paper</t>
+          <t>AMWAT Moving Warehousing Storage</t>
         </is>
       </c>
       <c r="B5" s="46" t="inlineStr">
@@ -2390,25 +2574,25 @@
       </c>
       <c r="C5" s="46" t="inlineStr">
         <is>
-          <t>Transportation, Logistics, Supply Chain and Storage</t>
+          <t>Warehousing and Storage</t>
         </is>
       </c>
       <c r="D5" s="46" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E5" s="46" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="F5" s="46" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G5" s="46" t="inlineStr">
         <is>
-          <t>Armando Caceres</t>
+          <t>Gloria Maria Pugh</t>
         </is>
       </c>
       <c r="H5" s="46" t="inlineStr">
@@ -2427,7 +2611,7 @@
         </is>
       </c>
       <c r="K5" s="49" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="L5" s="46" t="inlineStr">
         <is>
@@ -2435,16 +2619,16 @@
         </is>
       </c>
       <c r="M5" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="N5" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="46" t="inlineStr">
         <is>
-          <t>Acosta</t>
+          <t>All Florida Paper</t>
         </is>
       </c>
       <c r="B6" s="46" t="inlineStr">
@@ -2454,30 +2638,30 @@
       </c>
       <c r="C6" s="46" t="inlineStr">
         <is>
-          <t>Business Services &amp; Supplies</t>
+          <t>Transportation, Logistics, Supply Chain and Storage</t>
         </is>
       </c>
       <c r="D6" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E6" s="46" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="F6" s="46" t="n">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="G6" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Armando Caceres</t>
         </is>
       </c>
       <c r="H6" s="46" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I6" s="46" t="inlineStr">
@@ -2490,8 +2674,8 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K6" s="50" t="n">
-        <v>35</v>
+      <c r="K6" s="49" t="n">
+        <v>45</v>
       </c>
       <c r="L6" s="46" t="inlineStr">
         <is>
@@ -2508,17 +2692,17 @@
     <row r="7">
       <c r="A7" s="46" t="inlineStr">
         <is>
-          <t>Accordis International</t>
+          <t>Alternalight llc</t>
         </is>
       </c>
       <c r="B7" s="46" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C7" s="46" t="inlineStr">
         <is>
-          <t>IT Services and IT Consulting</t>
+          <t>Alternative Energy</t>
         </is>
       </c>
       <c r="D7" s="46" t="inlineStr">
@@ -2528,15 +2712,15 @@
       </c>
       <c r="E7" s="46" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="F7" s="46" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G7" s="46" t="inlineStr">
         <is>
-          <t>Rehan Khan</t>
+          <t>Russell Stidolph</t>
         </is>
       </c>
       <c r="H7" s="46" t="inlineStr">
@@ -2554,8 +2738,8 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K7" s="50" t="n">
-        <v>35</v>
+      <c r="K7" s="49" t="n">
+        <v>45</v>
       </c>
       <c r="L7" s="46" t="inlineStr">
         <is>
@@ -2563,26 +2747,26 @@
         </is>
       </c>
       <c r="M7" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="N7" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="46" t="inlineStr">
         <is>
-          <t>Accordion Partners</t>
+          <t>Ameritape, Inc.</t>
         </is>
       </c>
       <c r="B8" s="46" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="C8" s="46" t="inlineStr">
         <is>
-          <t>Consulting firm</t>
+          <t>Automation Machinery Manufacturing</t>
         </is>
       </c>
       <c r="D8" s="46" t="inlineStr">
@@ -2592,20 +2776,20 @@
       </c>
       <c r="E8" s="46" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>1990</t>
         </is>
       </c>
       <c r="F8" s="46" t="n">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="G8" s="46" t="inlineStr">
         <is>
-          <t>Nick Leopard</t>
+          <t>Renee Soares, Tom Whipple</t>
         </is>
       </c>
       <c r="H8" s="46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I8" s="46" t="inlineStr">
@@ -2618,8 +2802,8 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="K8" s="50" t="n">
-        <v>25</v>
+      <c r="K8" s="49" t="n">
+        <v>40</v>
       </c>
       <c r="L8" s="46" t="inlineStr">
         <is>
@@ -2627,26 +2811,26 @@
         </is>
       </c>
       <c r="M8" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="N8" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="46" t="inlineStr">
         <is>
-          <t>Allo</t>
+          <t>Accordis International</t>
         </is>
       </c>
       <c r="B9" s="46" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="C9" s="46" t="inlineStr">
         <is>
-          <t>Telecommunications</t>
+          <t>IT Services and IT Consulting</t>
         </is>
       </c>
       <c r="D9" s="46" t="inlineStr">
@@ -2656,20 +2840,20 @@
       </c>
       <c r="E9" s="46" t="inlineStr">
         <is>
-          <t>2003</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="F9" s="46" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G9" s="46" t="inlineStr">
         <is>
-          <t>Brad Moline</t>
+          <t>Rehan Khan</t>
         </is>
       </c>
       <c r="H9" s="46" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I9" s="46" t="inlineStr">
@@ -2683,7 +2867,7 @@
         </is>
       </c>
       <c r="K9" s="50" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="L9" s="46" t="inlineStr">
         <is>
@@ -2700,17 +2884,17 @@
     <row r="10">
       <c r="A10" s="46" t="inlineStr">
         <is>
-          <t>Accelerate Capital Group</t>
+          <t>Acosta</t>
         </is>
       </c>
       <c r="B10" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="C10" s="46" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Business Services &amp; Supplies</t>
         </is>
       </c>
       <c r="D10" s="46" t="inlineStr">
@@ -2720,20 +2904,20 @@
       </c>
       <c r="E10" s="46" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1927</t>
         </is>
       </c>
       <c r="F10" s="46" t="n">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="G10" s="46" t="inlineStr">
         <is>
-          <t>Alexis Graham, Ian Tracy</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H10" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I10" s="46" t="inlineStr">
@@ -2747,7 +2931,7 @@
         </is>
       </c>
       <c r="K10" s="50" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="L10" s="46" t="inlineStr">
         <is>
@@ -2764,31 +2948,31 @@
     <row r="11">
       <c r="A11" s="46" t="inlineStr">
         <is>
-          <t>2600Hz</t>
+          <t>AirQuest Environmental, Inc.</t>
         </is>
       </c>
       <c r="B11" s="46" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="C11" s="46" t="inlineStr">
         <is>
-          <t>Telecommunications</t>
+          <t>Environmental Services</t>
         </is>
       </c>
       <c r="D11" s="46" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E11" s="46" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="F11" s="46" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G11" s="46" t="inlineStr">
         <is>
@@ -2797,7 +2981,7 @@
       </c>
       <c r="H11" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I11" s="46" t="inlineStr">
@@ -2811,7 +2995,7 @@
         </is>
       </c>
       <c r="K11" s="50" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="L11" s="46" t="inlineStr">
         <is>
@@ -2819,49 +3003,49 @@
         </is>
       </c>
       <c r="M11" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="N11" s="48" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="46" t="inlineStr">
         <is>
-          <t>Affinity Beverages LLC</t>
+          <t>Accordion Partners</t>
         </is>
       </c>
       <c r="B12" s="46" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="C12" s="46" t="inlineStr">
         <is>
-          <t>Food &amp; Beverages</t>
+          <t>Consulting firm</t>
         </is>
       </c>
       <c r="D12" s="46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E12" s="46" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="F12" s="46" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G12" s="46" t="inlineStr">
         <is>
-          <t>Stanley Rottell</t>
+          <t>Nick Leopard</t>
         </is>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I12" s="46" t="inlineStr">
@@ -2875,7 +3059,7 @@
         </is>
       </c>
       <c r="K12" s="50" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="L12" s="46" t="inlineStr">
         <is>
@@ -2886,6 +3070,262 @@
         <v>46195</v>
       </c>
       <c r="N12" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>Allo</t>
+        </is>
+      </c>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Telecommunications</t>
+        </is>
+      </c>
+      <c r="D13" s="46" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="F13" s="46" t="n">
+        <v>23</v>
+      </c>
+      <c r="G13" s="46" t="inlineStr">
+        <is>
+          <t>Brad Moline</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I13" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J13" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K13" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="L13" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M13" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N13" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t>Affinity Beverages LLC</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>Stanley Rottell</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I14" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J14" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K14" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L14" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M14" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N14" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="46" t="inlineStr">
+        <is>
+          <t>Accelerate Capital Group</t>
+        </is>
+      </c>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="D15" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="F15" s="46" t="n">
+        <v>18</v>
+      </c>
+      <c r="G15" s="46" t="inlineStr">
+        <is>
+          <t>Alexis Graham, Ian Tracy</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I15" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J15" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K15" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L15" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M15" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N15" s="48" t="n">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="46" t="inlineStr">
+        <is>
+          <t>2600Hz</t>
+        </is>
+      </c>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>Telecommunications</t>
+        </is>
+      </c>
+      <c r="D16" s="46" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="F16" s="46" t="n">
+        <v>16</v>
+      </c>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I16" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="J16" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K16" s="50" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" s="46" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="M16" s="48" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N16" s="48" t="n">
         <v>46195</v>
       </c>
     </row>
@@ -3100,11 +3540,11 @@
       </c>
       <c r="B5" s="52" t="inlineStr">
         <is>
-          <t>All Florida Paper</t>
+          <t>AMWAT Moving Warehousing Storage</t>
         </is>
       </c>
       <c r="C5" s="54" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D5" s="52" t="inlineStr">
         <is>
@@ -3113,17 +3553,17 @@
       </c>
       <c r="E5" s="52" t="inlineStr">
         <is>
-          <t>All Florida Paper has a long-standing presence in the transportation, logistics, supply chain, and storage industry, having been founded in 1993. With 33 years in business, the company demonstrates stability and experience, making it a potentially attractive acquisition target.</t>
+          <t>AMWAT Moving Warehousing Storage is a strong acquisition target due to its long-standing presence in the industry, having been operational for over 25 years. The company is led by its founder, Gloria Maria Pugh, which may indicate stability and a strong vision for the business.</t>
         </is>
       </c>
       <c r="F5" s="52" t="inlineStr">
         <is>
-          <t>The Seller Readiness Score of 45 indicates a moderate level of preparedness for a sale, although no additional evidence is provided to further support this selection.</t>
+          <t>The company was founded in 1997 by Gloria Maria Pugh, who currently serves as President &amp; CEO, and is explicitly described as locally owned.</t>
         </is>
       </c>
       <c r="G5" s="52" t="inlineStr">
         <is>
-          <t>Established logistics company with 33 years of experience and moderate seller readiness.</t>
+          <t>Established warehousing company with over 25 years of operational experience.</t>
         </is>
       </c>
       <c r="H5" s="52" t="inlineStr">
@@ -3133,7 +3573,7 @@
       </c>
       <c r="I5" s="52" t="inlineStr"/>
       <c r="J5" s="52" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" ht="90" customHeight="1">
@@ -3142,11 +3582,11 @@
       </c>
       <c r="B6" s="52" t="inlineStr">
         <is>
-          <t>Acosta</t>
-        </is>
-      </c>
-      <c r="C6" s="55" t="n">
-        <v>35</v>
+          <t>All Florida Paper</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="n">
+        <v>45</v>
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
@@ -3155,17 +3595,17 @@
       </c>
       <c r="E6" s="52" t="inlineStr">
         <is>
-          <t>Acosta is a well-established company with 99 years in the business services and supplies industry, indicating stability and experience. The current leadership under CEO Darian Pickett suggests a potential for continued growth and innovation, making it an attractive acquisition target.</t>
+          <t>All Florida Paper has a long-standing presence in the transportation, logistics, supply chain, and storage industry, having been founded in 1993. With 33 years in business, the company demonstrates stability and experience, making it a potentially attractive acquisition target.</t>
         </is>
       </c>
       <c r="F6" s="52" t="inlineStr">
         <is>
-          <t>Acosta Sales &amp; Marketing was founded in 1927, and the current CEO is Darian Pickett, indicating a strong leadership structure. However, details about family ownership and the founder's background are limited.</t>
+          <t>The Seller Readiness Score of 45 indicates a moderate level of preparedness for a sale, although no additional evidence is provided to further support this selection.</t>
         </is>
       </c>
       <c r="G6" s="52" t="inlineStr">
         <is>
-          <t>Acosta's long history and current leadership make it a compelling acquisition target.</t>
+          <t>Established logistics company with 33 years of experience and moderate seller readiness.</t>
         </is>
       </c>
       <c r="H6" s="52" t="inlineStr">
@@ -3175,7 +3615,7 @@
       </c>
       <c r="I6" s="52" t="inlineStr"/>
       <c r="J6" s="52" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="90" customHeight="1">
@@ -3184,30 +3624,30 @@
       </c>
       <c r="B7" s="52" t="inlineStr">
         <is>
-          <t>Accordis International</t>
-        </is>
-      </c>
-      <c r="C7" s="55" t="n">
-        <v>35</v>
+          <t>Alternalight llc</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="n">
+        <v>45</v>
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E7" s="52" t="inlineStr">
         <is>
-          <t>Accordis International has been in business for 18 years, indicating stability and experience in the IT Services and IT Consulting industry. The founder-led structure may provide a strong vision and leadership continuity, making it an attractive acquisition target.</t>
+          <t>Alternalight LLC is a strong acquisition target due to its 20 years of experience in the alternative energy sector and its founder-led management under Russell Stidolph. The company's established presence and private ownership suggest potential for strategic growth and innovation in a rapidly evolving industry.</t>
         </is>
       </c>
       <c r="F7" s="52" t="inlineStr">
         <is>
-          <t>The evidence is limited, with no additional information captured, but the company's long tenure and founder-led status support its potential as an acquisition target.</t>
+          <t>The company was founded in 2006 by Russell Stidolph, who currently serves as Managing Director, indicating strong leadership continuity. The Seller Readiness Score of 45 suggests a moderate level of preparedness for acquisition.</t>
         </is>
       </c>
       <c r="G7" s="52" t="inlineStr">
         <is>
-          <t>Accordis International is a stable, experienced IT services firm with founder-led leadership.</t>
+          <t>Alternalight LLC offers 20 years of experience in alternative energy under strong founder leadership.</t>
         </is>
       </c>
       <c r="H7" s="52" t="inlineStr">
@@ -3217,7 +3657,7 @@
       </c>
       <c r="I7" s="52" t="inlineStr"/>
       <c r="J7" s="52" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1">
@@ -3226,30 +3666,30 @@
       </c>
       <c r="B8" s="52" t="inlineStr">
         <is>
-          <t>Accordion Partners</t>
-        </is>
-      </c>
-      <c r="C8" s="55" t="n">
-        <v>25</v>
+          <t>Ameritape, Inc.</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="n">
+        <v>40</v>
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E8" s="52" t="inlineStr">
         <is>
-          <t>Accordion Partners is a well-established consulting firm with 17 years in business, led by its founder Nick Leopard. The company's private status and the founder's active role as CEO suggest potential for strategic growth and alignment with acquisition goals.</t>
+          <t>Ameritape, Inc. is a well-established company with 36 years in the automation machinery manufacturing industry, indicating stability and experience. The company's focus on pressure-sensitive adhesive tape products positions it in a niche market, potentially attractive for strategic acquisition.</t>
         </is>
       </c>
       <c r="F8" s="52" t="inlineStr">
         <is>
-          <t>The company was founded in 2009 by Nick Leopard, who currently serves as CEO and Founder, indicating strong leadership. However, evidence regarding family ownership and the founder's age is limited.</t>
+          <t>Ameritape, Inc. was founded in 1990 and has been privately owned since two employees purchased it in 2008. The company currently employs 18 people, suggesting a manageable size for acquisition.</t>
         </is>
       </c>
       <c r="G8" s="52" t="inlineStr">
         <is>
-          <t>Accordion Partners is a seasoned consulting firm with strong leadership and growth potential.</t>
+          <t>Ameritape, Inc. is a stable, niche player in automation machinery manufacturing.</t>
         </is>
       </c>
       <c r="H8" s="52" t="inlineStr">
@@ -3259,7 +3699,7 @@
       </c>
       <c r="I8" s="52" t="inlineStr"/>
       <c r="J8" s="52" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
@@ -3268,30 +3708,30 @@
       </c>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>Allo</t>
+          <t>Accordis International</t>
         </is>
       </c>
       <c r="C9" s="55" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D9" s="52" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E9" s="52" t="inlineStr">
         <is>
-          <t>Allo is a well-established telecommunications company with 23 years in business, indicating stability and experience in the industry. Its Seller Readiness Score of 20 suggests a potential willingness to engage in acquisition discussions.</t>
+          <t>Accordis International has been in business for 18 years, indicating stability and experience in the IT Services and IT Consulting industry. The founder-led structure may provide a strong vision and leadership continuity, making it an attractive acquisition target.</t>
         </is>
       </c>
       <c r="F9" s="52" t="inlineStr">
         <is>
-          <t>Evidence is limited, but the company's long history and Seller Readiness Score support its selection as an acquisition target.</t>
+          <t>The evidence is limited, with no additional information captured, but the company's long tenure and founder-led status support its potential as an acquisition target.</t>
         </is>
       </c>
       <c r="G9" s="52" t="inlineStr">
         <is>
-          <t>Allo is a stable telecommunications company with a strong Seller Readiness Score.</t>
+          <t>Accordis International is a stable, experienced IT services firm with founder-led leadership.</t>
         </is>
       </c>
       <c r="H9" s="52" t="inlineStr">
@@ -3301,7 +3741,7 @@
       </c>
       <c r="I9" s="52" t="inlineStr"/>
       <c r="J9" s="52" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1">
@@ -3310,30 +3750,30 @@
       </c>
       <c r="B10" s="52" t="inlineStr">
         <is>
-          <t>Accelerate Capital Group</t>
+          <t>Acosta</t>
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E10" s="52" t="inlineStr">
         <is>
-          <t>Accelerate Capital Group has been in business for 18 years, indicating stability and experience in the financial services industry. The company has a high seller readiness score of 10, suggesting that it is well-prepared for acquisition discussions.</t>
+          <t>Acosta is a well-established company with 99 years in the business services and supplies industry, indicating stability and experience. The current leadership under CEO Darian Pickett suggests a potential for continued growth and innovation, making it an attractive acquisition target.</t>
         </is>
       </c>
       <c r="F10" s="52" t="inlineStr">
         <is>
-          <t>The evidence is limited, but the company's long tenure and high seller readiness score support its selection as an acquisition target.</t>
+          <t>Acosta Sales &amp; Marketing was founded in 1927, and the current CEO is Darian Pickett, indicating a strong leadership structure. However, details about family ownership and the founder's background are limited.</t>
         </is>
       </c>
       <c r="G10" s="52" t="inlineStr">
         <is>
-          <t>Accelerate Capital Group is a stable financial services firm with high seller readiness.</t>
+          <t>Acosta's long history and current leadership make it a compelling acquisition target.</t>
         </is>
       </c>
       <c r="H10" s="52" t="inlineStr">
@@ -3343,7 +3783,7 @@
       </c>
       <c r="I10" s="52" t="inlineStr"/>
       <c r="J10" s="52" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" ht="90" customHeight="1">
@@ -3352,30 +3792,30 @@
       </c>
       <c r="B11" s="52" t="inlineStr">
         <is>
-          <t>2600Hz</t>
+          <t>AirQuest Environmental, Inc.</t>
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D11" s="52" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="E11" s="52" t="inlineStr">
         <is>
-          <t>2600Hz is a strong acquisition target due to its established presence in the telecommunications industry, having been in business for 16 years. The company's high seller readiness score of 10 indicates a strong willingness to engage in a sale, making it an attractive option for potential buyers.</t>
+          <t>AirQuest Environmental, Inc. is a strong acquisition target due to its established presence in the environmental services industry, having been in business for 24 years. The company's niche focus on industrial hygiene and environmental consulting positions it well for growth and potential synergies with larger firms.</t>
         </is>
       </c>
       <c r="F11" s="52" t="inlineStr">
         <is>
-          <t>The evidence supporting this selection is limited, but the high seller readiness score of 10 is a significant indicator of the company's preparedness for acquisition.</t>
+          <t>AirQuest was incorporated in 2002 as a niche industrial hygiene and environmental consulting firm, indicating a specialized market presence. The Seller Readiness Score of 35 suggests a moderate level of preparedness for acquisition.</t>
         </is>
       </c>
       <c r="G11" s="52" t="inlineStr">
         <is>
-          <t>2600Hz is a prime acquisition target with a high seller readiness score.</t>
+          <t>Established environmental services firm with 24 years of niche expertise.</t>
         </is>
       </c>
       <c r="H11" s="52" t="inlineStr">
@@ -3385,7 +3825,7 @@
       </c>
       <c r="I11" s="52" t="inlineStr"/>
       <c r="J11" s="52" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>